<commit_message>
shiva mandir estimate complete and provided to upabhokta
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/nagar bhaipari and estimate misc/ढुंगाना गाउँ शिव मन्दिरको त्रस निर्माण/ढुंगाना गाउँ शिव मन्दिरको त्रस निर्माण.xlsx
+++ b/बजेट माग estimate/nagar bhaipari and estimate misc/ढुंगाना गाउँ शिव मन्दिरको त्रस निर्माण/ढुंगाना गाउँ शिव मन्दिरको त्रस निर्माण.xlsx
@@ -1,23 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D95B52D-CBCC-46D4-91F4-1E42B84A4AD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D31664-DFD7-4DCC-BDF0-1C186573EA62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="12" r:id="rId1"/>
+    <sheet name="estimate (2)" sheetId="13" r:id="rId2"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId2"/>
     <externalReference r:id="rId3"/>
     <externalReference r:id="rId4"/>
+    <externalReference r:id="rId5"/>
   </externalReferences>
   <definedNames>
     <definedName name="description_103">[1]Abstract!$B$16</definedName>
     <definedName name="description_124" localSheetId="0">#REF!</definedName>
+    <definedName name="description_124" localSheetId="1">#REF!</definedName>
     <definedName name="description_124">#REF!</definedName>
     <definedName name="description_247">[1]Abstract!$B$22</definedName>
     <definedName name="description_248">[1]Abstract!$B$23</definedName>
@@ -26,19 +28,25 @@
     <definedName name="description_276">[3]Abstract!$B$40</definedName>
     <definedName name="description_3">[1]Abstract!$B$169</definedName>
     <definedName name="description_310" localSheetId="0">#REF!</definedName>
+    <definedName name="description_310" localSheetId="1">#REF!</definedName>
     <definedName name="description_310">#REF!</definedName>
     <definedName name="description_312" localSheetId="0">#REF!</definedName>
+    <definedName name="description_312" localSheetId="1">#REF!</definedName>
     <definedName name="description_312">#REF!</definedName>
     <definedName name="description_5">[1]Abstract!$B$171</definedName>
     <definedName name="description_6" localSheetId="0">#REF!</definedName>
+    <definedName name="description_6" localSheetId="1">#REF!</definedName>
     <definedName name="description_6">#REF!</definedName>
     <definedName name="description_759">[1]Abstract!$B$278</definedName>
     <definedName name="description_781" localSheetId="0">#REF!</definedName>
+    <definedName name="description_781" localSheetId="1">#REF!</definedName>
     <definedName name="description_781">#REF!</definedName>
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="description_784">[3]Abstract!$B$300</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$61</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'estimate (2)'!$A$1:$K$59</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'estimate (2)'!$1:$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -58,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="70">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -242,6 +250,42 @@
   </si>
   <si>
     <t xml:space="preserve">Date:                  </t>
+  </si>
+  <si>
+    <t>-MS square pipe of 3" * 3" of 2mm thickness for vertical post</t>
+  </si>
+  <si>
+    <t>-MS square pipe of 1.5" * 1.5" of 1.6mm thickness for arch</t>
+  </si>
+  <si>
+    <t>-MS square pipe of 1.5" * 1.5" of 1.6mm thickness for purlin</t>
+  </si>
+  <si>
+    <t>-for roof</t>
+  </si>
+  <si>
+    <t>=@ ld=ld= Kn]g kmfO{j/ Unf; kftfn] 5fgf 5fpg] sfd</t>
+  </si>
+  <si>
+    <t>-13% VAT for fiber glass</t>
+  </si>
+  <si>
+    <t>-13% VAT for 8mm nut bolt</t>
+  </si>
+  <si>
+    <t>g/d k|sf/sf] Sn] / l;N6L df6f]df ;j} lsl;dsf] vGg] sfd</t>
+  </si>
+  <si>
+    <t>sfnf] kmnfd] kfO{ksf] 6«; agfO{ h8fg ug]{ tyf ljleGg ;fO{hsf] kmnfd] PËn km]lj|s]zg u/L k|fOd/ k]G6 ;lxt ug]{ sfd</t>
+  </si>
+  <si>
+    <t>-MS square pipe of 1" * 1" of 1 .2mm thickness for purlin</t>
+  </si>
+  <si>
+    <t>Equal angle of 35mm*35mm*2mm for bench</t>
+  </si>
+  <si>
+    <t>MS Flat bar of 20mm*5mm</t>
   </si>
 </sst>
 </file>
@@ -416,7 +460,7 @@
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -526,23 +570,12 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -563,10 +596,24 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1113,113 +1160,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
     </row>
     <row r="2" spans="1:18" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="57"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-      <c r="E4" s="47"/>
-      <c r="F4" s="47"/>
-      <c r="G4" s="47"/>
-      <c r="H4" s="47"/>
-      <c r="I4" s="47"/>
-      <c r="J4" s="47"/>
-      <c r="K4" s="47"/>
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
+      <c r="I4" s="57"/>
+      <c r="J4" s="57"/>
+      <c r="K4" s="57"/>
     </row>
     <row r="5" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="48" t="s">
+      <c r="A5" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="48"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
-      <c r="F5" s="48"/>
-      <c r="G5" s="48"/>
-      <c r="H5" s="48"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="48"/>
-      <c r="K5" s="48"/>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="58"/>
+      <c r="F5" s="58"/>
+      <c r="G5" s="58"/>
+      <c r="H5" s="58"/>
+      <c r="I5" s="58"/>
+      <c r="J5" s="58"/>
+      <c r="K5" s="58"/>
     </row>
     <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="43"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="43"/>
+      <c r="B6" s="53"/>
+      <c r="C6" s="53"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="44" t="s">
+      <c r="H6" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="44"/>
-      <c r="J6" s="44"/>
-      <c r="K6" s="44"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="54"/>
+      <c r="K6" s="54"/>
     </row>
     <row r="7" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="51" t="s">
+      <c r="A7" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="51"/>
-      <c r="C7" s="51"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="51"/>
+      <c r="B7" s="48"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="52" t="s">
+      <c r="H7" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="I7" s="52"/>
-      <c r="J7" s="52"/>
-      <c r="K7" s="52"/>
+      <c r="I7" s="49"/>
+      <c r="J7" s="49"/>
+      <c r="K7" s="49"/>
     </row>
     <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -1740,7 +1787,7 @@
         <f>B35</f>
         <v>-for plinth</v>
       </c>
-      <c r="C30" s="57">
+      <c r="C30" s="44">
         <v>0.5</v>
       </c>
       <c r="D30" s="33">
@@ -1767,7 +1814,7 @@
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="16"/>
       <c r="B31" s="32"/>
-      <c r="C31" s="57">
+      <c r="C31" s="44">
         <v>0.5</v>
       </c>
       <c r="D31" s="33">
@@ -2002,7 +2049,7 @@
       <c r="I41" s="17"/>
       <c r="J41" s="17"/>
       <c r="K41" s="17"/>
-      <c r="Q41" s="56"/>
+      <c r="Q41" s="43"/>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="16"/>
@@ -2293,11 +2340,11 @@
       <c r="B56" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C56" s="49">
+      <c r="C56" s="46">
         <f>J54</f>
         <v>200422.95926556629</v>
       </c>
-      <c r="D56" s="50"/>
+      <c r="D56" s="47"/>
       <c r="E56" s="9">
         <v>100</v>
       </c>
@@ -2319,21 +2366,21 @@
       <c r="B57" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="C57" s="53">
+      <c r="C57" s="50">
         <v>175000</v>
       </c>
-      <c r="D57" s="54"/>
+      <c r="D57" s="51"/>
       <c r="E57" s="9"/>
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B58" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C58" s="53">
+      <c r="C58" s="50">
         <f>C57-C60-C61</f>
         <v>166250</v>
       </c>
-      <c r="D58" s="54"/>
+      <c r="D58" s="51"/>
       <c r="E58" s="9">
         <f>C58/C56*100</f>
         <v>82.949578535917084</v>
@@ -2343,11 +2390,11 @@
       <c r="B59" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C59" s="55">
+      <c r="C59" s="52">
         <f>C56-C58</f>
         <v>34172.959265566285</v>
       </c>
-      <c r="D59" s="55"/>
+      <c r="D59" s="52"/>
       <c r="E59" s="9">
         <f>100-E58</f>
         <v>17.050421464082916</v>
@@ -2357,11 +2404,11 @@
       <c r="B60" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C60" s="49">
+      <c r="C60" s="46">
         <f>C57*0.03</f>
         <v>5250</v>
       </c>
-      <c r="D60" s="50"/>
+      <c r="D60" s="47"/>
       <c r="E60" s="9">
         <v>3</v>
       </c>
@@ -2370,17 +2417,24 @@
       <c r="B61" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C61" s="49">
+      <c r="C61" s="46">
         <f>C57*0.02</f>
         <v>3500</v>
       </c>
-      <c r="D61" s="50"/>
+      <c r="D61" s="47"/>
       <c r="E61" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C60:D60"/>
     <mergeCell ref="C61:D61"/>
     <mergeCell ref="A7:F7"/>
@@ -2389,6 +2443,1264 @@
     <mergeCell ref="C57:D57"/>
     <mergeCell ref="C58:D58"/>
     <mergeCell ref="C59:D59"/>
+  </mergeCells>
+  <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
+  <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02F46B58-807D-4329-8B5F-7E44966801E9}">
+  <dimension ref="A1:S59"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" style="19" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" style="19" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" style="19" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="19"/>
+    <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5703125" style="19" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="9.140625" style="19"/>
+    <col min="13" max="16" width="0" style="19" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="37.28515625" style="19" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="55" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+    </row>
+    <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="56" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="57" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="57"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="57" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
+      <c r="I4" s="57"/>
+      <c r="J4" s="57"/>
+      <c r="K4" s="57"/>
+    </row>
+    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="58" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="58"/>
+      <c r="F5" s="58"/>
+      <c r="G5" s="58"/>
+      <c r="H5" s="58"/>
+      <c r="I5" s="58"/>
+      <c r="J5" s="58"/>
+      <c r="K5" s="58"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="53" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="53"/>
+      <c r="C6" s="53"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="54"/>
+      <c r="J6" s="54"/>
+      <c r="K6" s="54"/>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="48"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="I7" s="49"/>
+      <c r="J7" s="49"/>
+      <c r="K7" s="49"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" s="34" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>1</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" s="37"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="38"/>
+      <c r="K9" s="5"/>
+    </row>
+    <row r="10" spans="1:11" s="34" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="16"/>
+      <c r="B10" s="39" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="40">
+        <v>9</v>
+      </c>
+      <c r="D10" s="9">
+        <f>(9+1)/3.281</f>
+        <v>3.047851264858275</v>
+      </c>
+      <c r="E10" s="9">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="F10" s="9">
+        <f t="shared" ref="F10:F12" si="0">PRODUCT(C10:E10)</f>
+        <v>120.69491008838769</v>
+      </c>
+      <c r="G10" s="9">
+        <f t="shared" ref="G10:G12" si="1">F10</f>
+        <v>120.69491008838769</v>
+      </c>
+      <c r="H10" s="38"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="38"/>
+      <c r="K10" s="27"/>
+    </row>
+    <row r="11" spans="1:11" s="34" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="16"/>
+      <c r="B11" s="39" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="40">
+        <v>6</v>
+      </c>
+      <c r="D11" s="9">
+        <f>11/3.281</f>
+        <v>3.3526363913441024</v>
+      </c>
+      <c r="E11" s="9">
+        <v>1.83</v>
+      </c>
+      <c r="F11" s="9">
+        <f t="shared" si="0"/>
+        <v>36.811947576958246</v>
+      </c>
+      <c r="G11" s="9">
+        <f t="shared" si="1"/>
+        <v>36.811947576958246</v>
+      </c>
+      <c r="H11" s="38"/>
+      <c r="I11" s="38"/>
+      <c r="J11" s="38"/>
+      <c r="K11" s="27"/>
+    </row>
+    <row r="12" spans="1:11" s="34" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="16"/>
+      <c r="B12" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="40">
+        <v>10</v>
+      </c>
+      <c r="D12" s="9">
+        <f>(35)/3.281</f>
+        <v>10.667479427003961</v>
+      </c>
+      <c r="E12" s="9">
+        <v>1.83</v>
+      </c>
+      <c r="F12" s="9">
+        <f t="shared" si="0"/>
+        <v>195.2148735141725</v>
+      </c>
+      <c r="G12" s="9">
+        <f t="shared" si="1"/>
+        <v>195.2148735141725</v>
+      </c>
+      <c r="H12" s="38"/>
+      <c r="I12" s="38"/>
+      <c r="J12" s="38"/>
+      <c r="K12" s="27"/>
+    </row>
+    <row r="13" spans="1:11" s="34" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="16"/>
+      <c r="B13" s="39" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="40">
+        <f>3*2</f>
+        <v>6</v>
+      </c>
+      <c r="D13" s="9">
+        <f>(2+2+1.33+2)/3.281</f>
+        <v>2.2340749771411152</v>
+      </c>
+      <c r="E13" s="9">
+        <v>1.04</v>
+      </c>
+      <c r="F13" s="9">
+        <f t="shared" ref="F13:F14" si="2">PRODUCT(C13:E13)</f>
+        <v>13.94062785736056</v>
+      </c>
+      <c r="G13" s="9">
+        <f t="shared" ref="G13:G14" si="3">F13</f>
+        <v>13.94062785736056</v>
+      </c>
+      <c r="H13" s="38"/>
+      <c r="I13" s="38"/>
+      <c r="J13" s="38"/>
+      <c r="K13" s="27"/>
+    </row>
+    <row r="14" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="16"/>
+      <c r="B14" s="39"/>
+      <c r="C14" s="40">
+        <f>2*3</f>
+        <v>6</v>
+      </c>
+      <c r="D14" s="9">
+        <f>10/3.281</f>
+        <v>3.047851264858275</v>
+      </c>
+      <c r="E14" s="9">
+        <v>1.04</v>
+      </c>
+      <c r="F14" s="9">
+        <f t="shared" si="2"/>
+        <v>19.018591892715637</v>
+      </c>
+      <c r="G14" s="9">
+        <f t="shared" si="3"/>
+        <v>19.018591892715637</v>
+      </c>
+      <c r="H14" s="38"/>
+      <c r="I14" s="38"/>
+      <c r="J14" s="38"/>
+      <c r="K14" s="27"/>
+    </row>
+    <row r="15" spans="1:11" s="34" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="16"/>
+      <c r="B15" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="40">
+        <f>2*2</f>
+        <v>4</v>
+      </c>
+      <c r="D15" s="9">
+        <f>10/3.281</f>
+        <v>3.047851264858275</v>
+      </c>
+      <c r="E15" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="F15" s="9">
+        <f t="shared" ref="F15:F16" si="4">PRODUCT(C15:E15)</f>
+        <v>10.97226455348979</v>
+      </c>
+      <c r="G15" s="9">
+        <f t="shared" ref="G15:G16" si="5">F15</f>
+        <v>10.97226455348979</v>
+      </c>
+      <c r="H15" s="38"/>
+      <c r="I15" s="38"/>
+      <c r="J15" s="38"/>
+      <c r="K15" s="27"/>
+    </row>
+    <row r="16" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="16"/>
+      <c r="B16" s="39"/>
+      <c r="C16" s="40">
+        <f>2*3</f>
+        <v>6</v>
+      </c>
+      <c r="D16" s="9">
+        <f>1.25/3.281</f>
+        <v>0.38098140810728437</v>
+      </c>
+      <c r="E16" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="F16" s="9">
+        <f t="shared" si="4"/>
+        <v>2.0572996037793354</v>
+      </c>
+      <c r="G16" s="9">
+        <f t="shared" si="5"/>
+        <v>2.0572996037793354</v>
+      </c>
+      <c r="H16" s="38"/>
+      <c r="I16" s="38"/>
+      <c r="J16" s="38"/>
+      <c r="K16" s="27"/>
+    </row>
+    <row r="17" spans="1:17" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="16"/>
+      <c r="B17" s="39" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="40">
+        <v>13</v>
+      </c>
+      <c r="D17" s="9">
+        <f>10/3.281</f>
+        <v>3.047851264858275</v>
+      </c>
+      <c r="E17" s="9">
+        <v>0.78</v>
+      </c>
+      <c r="F17" s="9">
+        <f t="shared" ref="F17" si="6">PRODUCT(C17:E17)</f>
+        <v>30.905211825662906</v>
+      </c>
+      <c r="G17" s="9">
+        <f t="shared" ref="G17" si="7">F17</f>
+        <v>30.905211825662906</v>
+      </c>
+      <c r="H17" s="38"/>
+      <c r="I17" s="38"/>
+      <c r="J17" s="38"/>
+      <c r="K17" s="27"/>
+    </row>
+    <row r="18" spans="1:17" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="38">
+        <f>SUM(G10:G17)</f>
+        <v>429.61572691252655</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I18" s="6">
+        <v>182.51</v>
+      </c>
+      <c r="J18" s="38">
+        <f>G18*I18</f>
+        <v>78409.166318805219</v>
+      </c>
+      <c r="K18" s="5"/>
+    </row>
+    <row r="19" spans="1:17" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="39" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="3"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="38"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="38">
+        <f>0.13*G18*(1871.42/18.94)</f>
+        <v>5518.4208170867614</v>
+      </c>
+      <c r="K19" s="5"/>
+    </row>
+    <row r="20" spans="1:17" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="39"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="38"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="38"/>
+      <c r="K20" s="5"/>
+    </row>
+    <row r="21" spans="1:17" s="34" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>2</v>
+      </c>
+      <c r="B21" s="45" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="3"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="38"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="38"/>
+      <c r="K21" s="5"/>
+    </row>
+    <row r="22" spans="1:17" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="39" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="3">
+        <v>1</v>
+      </c>
+      <c r="D22" s="4">
+        <f>35/3.281</f>
+        <v>10.667479427003961</v>
+      </c>
+      <c r="E22" s="5">
+        <f>11/3.281</f>
+        <v>3.3526363913441024</v>
+      </c>
+      <c r="F22" s="5"/>
+      <c r="G22" s="33">
+        <f t="shared" ref="G22" si="8">PRODUCT(C22:F22)</f>
+        <v>35.764179730888017</v>
+      </c>
+      <c r="H22" s="7"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="38"/>
+      <c r="K22" s="5"/>
+    </row>
+    <row r="23" spans="1:17" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="3"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="38">
+        <f>SUM(G22:G22)</f>
+        <v>35.764179730888017</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I23" s="6">
+        <v>2150.64</v>
+      </c>
+      <c r="J23" s="38">
+        <f>G23*I23</f>
+        <v>76915.875496437002</v>
+      </c>
+      <c r="K23" s="5"/>
+      <c r="Q23" s="19"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A24" s="16"/>
+      <c r="B24" s="32" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="18">
+        <f>0.13*G23*17431.2/10</f>
+        <v>8104.3634064257185</v>
+      </c>
+      <c r="K24" s="17"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A25" s="16"/>
+      <c r="B25" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="18">
+        <f>0.13*G23*1023.75/10</f>
+        <v>475.97652699345599</v>
+      </c>
+      <c r="K25" s="17"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A26" s="16"/>
+      <c r="B26" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="18">
+        <f>0.13*G23*348.21/10</f>
+        <v>161.8947853132027</v>
+      </c>
+      <c r="K26" s="17"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A27" s="16"/>
+      <c r="B27" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="18">
+        <f>0.13*G23*165/10</f>
+        <v>76.714165522754811</v>
+      </c>
+      <c r="K27" s="17"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A28" s="16"/>
+      <c r="B28" s="32"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="18"/>
+      <c r="K28" s="17"/>
+    </row>
+    <row r="29" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="16">
+        <v>3</v>
+      </c>
+      <c r="B29" s="45" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="18"/>
+      <c r="K29" s="17"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A30" s="16"/>
+      <c r="B30" s="32" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="17">
+        <v>3</v>
+      </c>
+      <c r="D30" s="33">
+        <v>0.45</v>
+      </c>
+      <c r="E30" s="33">
+        <v>0.45</v>
+      </c>
+      <c r="F30" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="G30" s="33">
+        <f t="shared" ref="G30:G31" si="9">PRODUCT(C30:F30)</f>
+        <v>0.36449999999999999</v>
+      </c>
+      <c r="H30" s="17"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="18"/>
+      <c r="K30" s="17"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A31" s="16"/>
+      <c r="B31" s="32" t="str">
+        <f>B35</f>
+        <v>-for plinth</v>
+      </c>
+      <c r="C31" s="44">
+        <v>0.5</v>
+      </c>
+      <c r="D31" s="33">
+        <f>D35</f>
+        <v>5.6385248399878085</v>
+      </c>
+      <c r="E31" s="33">
+        <f>E35</f>
+        <v>2.3620847302651629</v>
+      </c>
+      <c r="F31" s="33">
+        <f>F35</f>
+        <v>0.15</v>
+      </c>
+      <c r="G31" s="33">
+        <f t="shared" si="9"/>
+        <v>0.99890050693170163</v>
+      </c>
+      <c r="H31" s="17"/>
+      <c r="I31" s="17"/>
+      <c r="J31" s="18"/>
+      <c r="K31" s="17"/>
+      <c r="Q31" s="34"/>
+    </row>
+    <row r="32" spans="1:17" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+      <c r="B32" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" s="3"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="38">
+        <f>SUM(G30:G31)</f>
+        <v>1.3634005069317017</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="I32" s="6">
+        <v>674.12</v>
+      </c>
+      <c r="J32" s="38">
+        <f>G32*I32</f>
+        <v>919.09554973279876</v>
+      </c>
+      <c r="K32" s="5"/>
+      <c r="Q32" s="19"/>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A33" s="16"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="17"/>
+      <c r="J33" s="18"/>
+      <c r="K33" s="17"/>
+    </row>
+    <row r="34" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="16">
+        <v>4</v>
+      </c>
+      <c r="B34" s="41" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="17"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="17"/>
+      <c r="J34" s="18"/>
+      <c r="K34" s="17"/>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A35" s="16"/>
+      <c r="B35" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="C35" s="17">
+        <v>1</v>
+      </c>
+      <c r="D35" s="33">
+        <f>18.5/3.281</f>
+        <v>5.6385248399878085</v>
+      </c>
+      <c r="E35" s="33">
+        <f>((8.5+7)/2)/3.281</f>
+        <v>2.3620847302651629</v>
+      </c>
+      <c r="F35" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G35" s="33">
+        <f t="shared" ref="G35:G36" si="10">PRODUCT(C35:F35)</f>
+        <v>1.9978010138634033</v>
+      </c>
+      <c r="H35" s="17"/>
+      <c r="I35" s="17"/>
+      <c r="J35" s="18"/>
+      <c r="K35" s="17"/>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A36" s="16"/>
+      <c r="B36" s="32" t="str">
+        <f>B30</f>
+        <v>-for footing of vertical post</v>
+      </c>
+      <c r="C36" s="17">
+        <f>C30</f>
+        <v>3</v>
+      </c>
+      <c r="D36" s="33">
+        <f>D30</f>
+        <v>0.45</v>
+      </c>
+      <c r="E36" s="33">
+        <f>E30</f>
+        <v>0.45</v>
+      </c>
+      <c r="F36" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G36" s="33">
+        <f t="shared" si="10"/>
+        <v>9.1124999999999998E-2</v>
+      </c>
+      <c r="H36" s="17"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="18"/>
+      <c r="K36" s="17"/>
+      <c r="Q36" s="34"/>
+    </row>
+    <row r="37" spans="1:17" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2"/>
+      <c r="B37" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="C37" s="3"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="38">
+        <f>SUM(G35:G36)</f>
+        <v>2.0889260138634032</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="I37" s="6">
+        <v>4458.5200000000004</v>
+      </c>
+      <c r="J37" s="38">
+        <f>G37*I37</f>
+        <v>9313.5184113302603</v>
+      </c>
+      <c r="K37" s="5"/>
+      <c r="Q37" s="19"/>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A38" s="16"/>
+      <c r="B38" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="17"/>
+      <c r="H38" s="17"/>
+      <c r="I38" s="17"/>
+      <c r="J38" s="18">
+        <f>0.13*G37*15452.64/5</f>
+        <v>839.2649636505206</v>
+      </c>
+      <c r="K38" s="17"/>
+    </row>
+    <row r="39" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="16"/>
+      <c r="B39" s="41"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
+      <c r="G39" s="17"/>
+      <c r="H39" s="17"/>
+      <c r="I39" s="17"/>
+      <c r="J39" s="18"/>
+      <c r="K39" s="17"/>
+      <c r="Q39" s="43"/>
+    </row>
+    <row r="40" spans="1:17" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="16">
+        <v>5</v>
+      </c>
+      <c r="B40" s="42" t="s">
+        <v>55</v>
+      </c>
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="17"/>
+      <c r="G40" s="17"/>
+      <c r="H40" s="17"/>
+      <c r="I40" s="17"/>
+      <c r="J40" s="17"/>
+      <c r="K40" s="17"/>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A41" s="16"/>
+      <c r="B41" s="32" t="str">
+        <f t="shared" ref="B41:E42" si="11">B35</f>
+        <v>-for plinth</v>
+      </c>
+      <c r="C41" s="17">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+      <c r="D41" s="33">
+        <f t="shared" si="11"/>
+        <v>5.6385248399878085</v>
+      </c>
+      <c r="E41" s="33">
+        <f t="shared" si="11"/>
+        <v>2.3620847302651629</v>
+      </c>
+      <c r="F41" s="33">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G41" s="33">
+        <f t="shared" ref="G41:G42" si="12">PRODUCT(C41:F41)</f>
+        <v>0.99890050693170163</v>
+      </c>
+      <c r="H41" s="17"/>
+      <c r="I41" s="17"/>
+      <c r="J41" s="18"/>
+      <c r="K41" s="17"/>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A42" s="16"/>
+      <c r="B42" s="32" t="str">
+        <f t="shared" si="11"/>
+        <v>-for footing of vertical post</v>
+      </c>
+      <c r="C42" s="17">
+        <f t="shared" si="11"/>
+        <v>3</v>
+      </c>
+      <c r="D42" s="33">
+        <f t="shared" si="11"/>
+        <v>0.45</v>
+      </c>
+      <c r="E42" s="33">
+        <f t="shared" si="11"/>
+        <v>0.45</v>
+      </c>
+      <c r="F42" s="33">
+        <f>0.05+0.3</f>
+        <v>0.35</v>
+      </c>
+      <c r="G42" s="33">
+        <f t="shared" si="12"/>
+        <v>0.21262500000000001</v>
+      </c>
+      <c r="H42" s="17"/>
+      <c r="I42" s="17"/>
+      <c r="J42" s="18"/>
+      <c r="K42" s="17"/>
+      <c r="Q42" s="34"/>
+    </row>
+    <row r="43" spans="1:17" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2"/>
+      <c r="B43" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="C43" s="3"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="38">
+        <f>SUM(G41:G42)</f>
+        <v>1.2115255069317017</v>
+      </c>
+      <c r="H43" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="I43" s="6">
+        <v>10964.46</v>
+      </c>
+      <c r="J43" s="38">
+        <f>G43*I43</f>
+        <v>13283.722959732364</v>
+      </c>
+      <c r="K43" s="5"/>
+      <c r="Q43" s="19"/>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A44" s="16"/>
+      <c r="B44" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="17"/>
+      <c r="F44" s="17"/>
+      <c r="G44" s="17"/>
+      <c r="H44" s="17"/>
+      <c r="I44" s="17"/>
+      <c r="J44" s="18">
+        <f>0.13*G43*53818.03/15</f>
+        <v>565.08327267440131</v>
+      </c>
+      <c r="K44" s="17"/>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A45" s="16"/>
+      <c r="B45" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="C45" s="17"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="17"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="17"/>
+      <c r="H45" s="17"/>
+      <c r="I45" s="17"/>
+      <c r="J45" s="18">
+        <f>0.13*G43*21432.6/15</f>
+        <v>225.03989369215805</v>
+      </c>
+      <c r="K45" s="17"/>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A46" s="16"/>
+      <c r="B46" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="C46" s="17"/>
+      <c r="D46" s="17"/>
+      <c r="E46" s="17"/>
+      <c r="F46" s="17"/>
+      <c r="G46" s="17"/>
+      <c r="H46" s="17"/>
+      <c r="I46" s="17"/>
+      <c r="J46" s="18">
+        <f>0.13*G43*(25719.12+13573.98+4286.52)/15</f>
+        <v>457.58111717405467</v>
+      </c>
+      <c r="K46" s="17"/>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A47" s="16"/>
+      <c r="B47" s="32" t="s">
+        <v>46</v>
+      </c>
+      <c r="C47" s="17"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="17"/>
+      <c r="F47" s="17"/>
+      <c r="G47" s="17"/>
+      <c r="H47" s="17"/>
+      <c r="I47" s="17"/>
+      <c r="J47" s="18">
+        <f>0.13*G43*(6325.7/15)</f>
+        <v>66.419139793048174</v>
+      </c>
+      <c r="K47" s="17"/>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A48" s="16"/>
+      <c r="B48" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C48" s="17"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="17"/>
+      <c r="F48" s="17"/>
+      <c r="G48" s="17"/>
+      <c r="H48" s="17"/>
+      <c r="I48" s="17"/>
+      <c r="J48" s="18">
+        <f>0.13*G43*(310)/5</f>
+        <v>9.7648955858695157</v>
+      </c>
+      <c r="K48" s="17"/>
+    </row>
+    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A49" s="16"/>
+      <c r="B49" s="32"/>
+      <c r="C49" s="17"/>
+      <c r="D49" s="17"/>
+      <c r="E49" s="17"/>
+      <c r="F49" s="17"/>
+      <c r="G49" s="17"/>
+      <c r="H49" s="17"/>
+      <c r="I49" s="17"/>
+      <c r="J49" s="18"/>
+      <c r="K49" s="17"/>
+    </row>
+    <row r="50" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="2">
+        <v>6</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C50" s="3">
+        <v>1</v>
+      </c>
+      <c r="D50" s="4"/>
+      <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="7">
+        <f t="shared" ref="G50" si="13">PRODUCT(C50:F50)</f>
+        <v>1</v>
+      </c>
+      <c r="H50" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I50" s="6">
+        <v>500</v>
+      </c>
+      <c r="J50" s="7">
+        <f>G50*I50</f>
+        <v>500</v>
+      </c>
+      <c r="K50" s="5"/>
+    </row>
+    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A51" s="2"/>
+      <c r="B51" s="8"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="6"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="6"/>
+      <c r="J51" s="18"/>
+      <c r="K51" s="5"/>
+    </row>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A52" s="21"/>
+      <c r="B52" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="C52" s="23"/>
+      <c r="D52" s="24"/>
+      <c r="E52" s="24"/>
+      <c r="F52" s="24"/>
+      <c r="G52" s="18"/>
+      <c r="H52" s="18"/>
+      <c r="I52" s="18"/>
+      <c r="J52" s="18">
+        <f>SUM(J9:J50)</f>
+        <v>195841.90171994959</v>
+      </c>
+      <c r="K52" s="25"/>
+      <c r="Q52" s="20"/>
+    </row>
+    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="M53" s="20"/>
+      <c r="N53" s="20"/>
+      <c r="O53" s="20"/>
+      <c r="P53" s="20"/>
+      <c r="R53" s="20"/>
+      <c r="S53" s="20"/>
+    </row>
+    <row r="54" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="26"/>
+      <c r="B54" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="C54" s="46">
+        <f>J52</f>
+        <v>195841.90171994959</v>
+      </c>
+      <c r="D54" s="47"/>
+      <c r="E54" s="9">
+        <v>100</v>
+      </c>
+      <c r="F54" s="26"/>
+      <c r="G54" s="28"/>
+      <c r="H54" s="26"/>
+      <c r="I54" s="29"/>
+      <c r="J54" s="30"/>
+      <c r="K54" s="31"/>
+      <c r="M54" s="19"/>
+      <c r="N54" s="19"/>
+      <c r="O54" s="19"/>
+      <c r="P54" s="19"/>
+      <c r="Q54" s="19"/>
+      <c r="R54" s="19"/>
+      <c r="S54" s="19"/>
+    </row>
+    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B55" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C55" s="50">
+        <v>175000</v>
+      </c>
+      <c r="D55" s="51"/>
+      <c r="E55" s="9"/>
+    </row>
+    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B56" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="C56" s="50">
+        <f>C55-C58-C59</f>
+        <v>166250</v>
+      </c>
+      <c r="D56" s="51"/>
+      <c r="E56" s="9">
+        <f>C56/C54*100</f>
+        <v>84.889902794007028</v>
+      </c>
+    </row>
+    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B57" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="C57" s="52">
+        <f>C54-C56</f>
+        <v>29591.901719949587</v>
+      </c>
+      <c r="D57" s="52"/>
+      <c r="E57" s="9">
+        <f>100-E56</f>
+        <v>15.110097205992972</v>
+      </c>
+    </row>
+    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B58" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="C58" s="46">
+        <f>C55*0.03</f>
+        <v>5250</v>
+      </c>
+      <c r="D58" s="47"/>
+      <c r="E58" s="9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B59" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="C59" s="46">
+        <f>C55*0.02</f>
+        <v>3500</v>
+      </c>
+      <c r="D59" s="47"/>
+      <c r="E59" s="9">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="C58:D58"/>
+    <mergeCell ref="C59:D59"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="C55:D55"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="C57:D57"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
@@ -2402,5 +3714,8 @@
   <headerFooter>
     <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
   </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="39" max="10" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
</xml_diff>